<commit_message>
ddPCR: réplicas biológicas por separado (E1 y E2), normalizadas vs media del c- y vs c- de la misma réplica
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0155wDXPt23zL2HdRwb5YjmM
</commit_message>
<xml_diff>
--- a/analisis/ddpcr_resultados.xlsx
+++ b/analisis/ddpcr_resultados.xlsx
@@ -9,15 +9,16 @@
   <sheets>
     <sheet name="Leeme" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Resumen global" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="E1 Pocillos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="E1 Medias" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="E1 Normalizado" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="E1 Resumen" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="E1 Gráficas" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="E2 Pocillos" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="E2 Medias" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="E2 Normalizado" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="E2 Gráficas" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Réplicas por separado" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="E1 Pocillos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="E1 Medias" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="E1 Normalizado" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="E1 Resumen" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="E1 Gráficas" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="E2 Pocillos" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="E2 Medias" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="E2 Normalizado" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="E2 Gráficas" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -72,12 +73,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -155,6 +159,86 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6096000" cy="4486275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>11</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6096000" cy="4486275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>59</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6096000" cy="4486275"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -559,7 +643,7 @@
 </wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
@@ -1172,7 +1256,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HOJAS:  E1 = experimento 01-oct (WT2 y MUT1)  ·  E2 = experimento 08-oct (solo MUT1)  ·  Resumen global = comparación de ambos.</t>
+          <t>HOJAS:  «Réplicas por separado» = cada réplica biológica sin promediar (E1 y E2)  ·  E1 = experimento 01-oct (WT2 y MUT1)  ·  E2 = experimento 08-oct (solo MUT1)  ·  Resumen global = comparación de ambos.</t>
         </is>
       </c>
     </row>
@@ -1275,6 +1359,604 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Sin corregir · por réplica biológica (media de las técnicas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Condicion</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Rep_bio</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>n_tecnicas</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>sd_tecnica</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>pocillos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2508.988</v>
+      </c>
+      <c r="E3" t="n">
+        <v>83.069</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>A01,A02</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1919.182</v>
+      </c>
+      <c r="E4" t="n">
+        <v>111.803</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>A03,A04</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>2</v>
+      </c>
+      <c r="D5" t="n">
+        <v>707.25</v>
+      </c>
+      <c r="E5" t="n">
+        <v>104.331</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>A05,A06</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1829.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>62.859</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>A07,A08</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>1366.621</v>
+      </c>
+      <c r="E7" t="n">
+        <v>76.241</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>A09,A10</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2</v>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1737.055</v>
+      </c>
+      <c r="E8" t="n">
+        <v>194.166</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>A11,A12</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Sin corregir · por condición (media ± SD de las 2 biológicas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Condicion</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>minimo</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>2214.085</v>
+      </c>
+      <c r="D12" t="n">
+        <v>417.056</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1919.182</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2508.988</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1551.838</v>
+      </c>
+      <c r="D13" t="n">
+        <v>261.936</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1366.621</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1737.055</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1268.225</v>
+      </c>
+      <c r="D14" t="n">
+        <v>793.338</v>
+      </c>
+      <c r="E14" t="n">
+        <v>707.25</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1829.2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Corregido por RNA · por réplica biológica (media de las técnicas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Condicion</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Rep_bio</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>n_tecnicas</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>sd_tecnica</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>pocillos</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="C18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" t="n">
+        <v>3584.269</v>
+      </c>
+      <c r="E18" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>A01,A02</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2</v>
+      </c>
+      <c r="C19" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" t="n">
+        <v>3095.455</v>
+      </c>
+      <c r="E19" t="n">
+        <v>180.327</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>A03,A04</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>1</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1360.097</v>
+      </c>
+      <c r="E20" t="n">
+        <v>200.637</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>A05,A06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" t="n">
+        <v>2286.5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>78.574</v>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>A07,A08</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" t="n">
+        <v>2</v>
+      </c>
+      <c r="D22" t="n">
+        <v>2628.117</v>
+      </c>
+      <c r="E22" t="n">
+        <v>146.617</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>A09,A10</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2198.804</v>
+      </c>
+      <c r="E23" t="n">
+        <v>245.78</v>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>A11,A12</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Corregido por RNA · por condición (media ± SD de las 2 biológicas)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Condicion</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>sd</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>minimo</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>maximo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="n">
+        <v>3339.862</v>
+      </c>
+      <c r="D27" t="n">
+        <v>345.644</v>
+      </c>
+      <c r="E27" t="n">
+        <v>3095.455</v>
+      </c>
+      <c r="F27" t="n">
+        <v>3584.269</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C28" t="n">
+        <v>2413.46</v>
+      </c>
+      <c r="D28" t="n">
+        <v>303.57</v>
+      </c>
+      <c r="E28" t="n">
+        <v>2198.804</v>
+      </c>
+      <c r="F28" t="n">
+        <v>2628.117</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>2</v>
+      </c>
+      <c r="C29" t="n">
+        <v>1823.299</v>
+      </c>
+      <c r="D29" t="n">
+        <v>655.066</v>
+      </c>
+      <c r="E29" t="n">
+        <v>1360.097</v>
+      </c>
+      <c r="F29" t="n">
+        <v>2286.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1539,7 +2221,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1998,6 +2680,1286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:R23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="17" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Cada réplica biológica por separado (no la media). 'Misma réplica' asume que la réplica 1 se aparea con el c- 1 y la 2 con el c- 2. E2: media de los 2 pocillos técnicos. E1: cada pocillo = una réplica (1 = primer pocillo).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="75" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Experimento</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Genotipo</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Condición</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>Réplica biológica</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>Pocillos</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Copias/µL</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>RNA</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Unid. RNA</t>
+        </is>
+      </c>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>Copias/µL ÷ RNA</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>SIN CORREGIR · veces vs MEDIA c-</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>SIN CORREGIR · veces vs c- MISMA réplica</t>
+        </is>
+      </c>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>SIN CORREGIR · veces MENOS vs media c- (1/x)</t>
+        </is>
+      </c>
+      <c r="M3" s="5" t="inlineStr">
+        <is>
+          <t>SIN CORREGIR · veces MENOS vs c- misma réplica (1/x)</t>
+        </is>
+      </c>
+      <c r="N3" s="5" t="inlineStr">
+        <is>
+          <t>POR RNA · veces vs MEDIA c-</t>
+        </is>
+      </c>
+      <c r="O3" s="5" t="inlineStr">
+        <is>
+          <t>POR RNA · veces vs c- MISMA réplica</t>
+        </is>
+      </c>
+      <c r="P3" s="5" t="inlineStr">
+        <is>
+          <t>POR RNA · veces MENOS vs media c- (1/x)</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>POR RNA · veces MENOS vs c- misma réplica (1/x)</t>
+        </is>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>Nota</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>A11</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>3986.943</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>2712.206</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1.254</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0.798</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="n">
+        <v>1.146</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.872</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>A12</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2373.573</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1.175</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>2020.062</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.746</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1.34</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.854</v>
+      </c>
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
+        <v>1.171</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>A07</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>2473.389</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1766.706</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1.286</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1.612</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.747</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.651</v>
+      </c>
+      <c r="P6" t="n">
+        <v>1.339</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>1.535</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>A08</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>1534.748</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1.53</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>1003.104</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.483</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0.647</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2.072</v>
+      </c>
+      <c r="M7" t="n">
+        <v>1.547</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.424</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.497</v>
+      </c>
+      <c r="P7" t="n">
+        <v>2.359</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>2.014</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>A05</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1497.313</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>1237.449</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.471</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0.376</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2.124</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2.663</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0.523</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.456</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1.912</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>2.192</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>A06</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>26.548</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>25.284</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.008</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="L9" t="n">
+        <v>119.794</v>
+      </c>
+      <c r="M9" t="n">
+        <v>89.408</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="P9" t="n">
+        <v>93.584</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>79.89700000000001</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>atípico (¿fallo técnico?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>WT2</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>A09</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>1247.478</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>840.053</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.8110000000000001</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1.233</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.859</v>
+      </c>
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>1.164</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>WT2</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>A10</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1828.767</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>1115.102</v>
+      </c>
+      <c r="J11" t="n">
+        <v>1.189</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0.841</v>
+      </c>
+      <c r="M11" t="n">
+        <v>1</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1.141</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.877</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>WT2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>A03</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1744.123</v>
+      </c>
+      <c r="G12" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>1194.605</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1.134</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1.398</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0.715</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1.222</v>
+      </c>
+      <c r="O12" t="n">
+        <v>1.422</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.8179999999999999</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.703</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>WT2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>A04</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>1775.182</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>1056.656</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1.154</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0.971</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1.081</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.948</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.925</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>1.055</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>WT2</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>A01</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>1531.069</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1020.712</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.995</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1.227</v>
+      </c>
+      <c r="L14" t="n">
+        <v>1.005</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0.8149999999999999</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1.044</v>
+      </c>
+      <c r="O14" t="n">
+        <v>1.215</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.958</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0.823</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>E1 (01-oct)</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>WT2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>A02</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>1151.032</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>µL</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>885.409</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.748</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0.629</v>
+      </c>
+      <c r="L15" t="n">
+        <v>1.336</v>
+      </c>
+      <c r="M15" t="n">
+        <v>1.589</v>
+      </c>
+      <c r="N15" t="n">
+        <v>0.906</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.794</v>
+      </c>
+      <c r="P15" t="n">
+        <v>1.104</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.259</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E2 (08-oct)</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>A01,A02</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>2508.989</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>ng/µL</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>3584.269</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1.133</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0.882</v>
+      </c>
+      <c r="M16" t="n">
+        <v>1</v>
+      </c>
+      <c r="N16" t="n">
+        <v>1.073</v>
+      </c>
+      <c r="O16" t="n">
+        <v>1</v>
+      </c>
+      <c r="P16" t="n">
+        <v>0.9320000000000001</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E2 (08-oct)</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>c-</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>A03,A04</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1919.182</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ng/µL</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>3095.455</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.867</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1.154</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1.079</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E2 (08-oct)</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>A09,A10</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>1366.621</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>ng/µL</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>2628.117</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.545</v>
+      </c>
+      <c r="L18" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="M18" t="n">
+        <v>1.836</v>
+      </c>
+      <c r="N18" t="n">
+        <v>0.787</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0.733</v>
+      </c>
+      <c r="P18" t="n">
+        <v>1.271</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1.364</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E2 (08-oct)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>#13 0,5NM</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>A11,A12</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1737.055</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>ng/µL</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>2198.804</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.784</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1.275</v>
+      </c>
+      <c r="M19" t="n">
+        <v>1.105</v>
+      </c>
+      <c r="N19" t="n">
+        <v>0.658</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0.71</v>
+      </c>
+      <c r="P19" t="n">
+        <v>1.519</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>1.408</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E2 (08-oct)</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>A05,A06</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>707.25</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>ng/µL</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1360.097</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.319</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3.131</v>
+      </c>
+      <c r="M20" t="n">
+        <v>3.547</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.407</v>
+      </c>
+      <c r="O20" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="P20" t="n">
+        <v>2.456</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>2.635</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E2 (08-oct)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MUT1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>#13 1NM</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>A07,A08</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1829.2</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>ng/µL</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>2286.5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.826</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.953</v>
+      </c>
+      <c r="L21" t="n">
+        <v>1.21</v>
+      </c>
+      <c r="M21" t="n">
+        <v>1.049</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.6850000000000001</v>
+      </c>
+      <c r="O21" t="n">
+        <v>0.739</v>
+      </c>
+      <c r="P21" t="n">
+        <v>1.461</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>1.354</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Gráficas (barra = réplica biológica; entre paréntesis ÷ = veces menos)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2700,7 +4662,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3682,7 +5644,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4609,7 +6571,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4766,7 +6728,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4816,7 +6778,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5622,602 +7584,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="3" t="inlineStr">
-        <is>
-          <t>Sin corregir · por réplica biológica (media de las técnicas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Condicion</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>Rep_bio</t>
-        </is>
-      </c>
-      <c r="C2" s="4" t="inlineStr">
-        <is>
-          <t>n_tecnicas</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>sd_tecnica</t>
-        </is>
-      </c>
-      <c r="F2" s="4" t="inlineStr">
-        <is>
-          <t>pocillos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>c-</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" t="n">
-        <v>2508.988</v>
-      </c>
-      <c r="E3" t="n">
-        <v>83.069</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>A01,A02</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>c-</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" t="n">
-        <v>1919.182</v>
-      </c>
-      <c r="E4" t="n">
-        <v>111.803</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>A03,A04</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>#13 1NM</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>2</v>
-      </c>
-      <c r="D5" t="n">
-        <v>707.25</v>
-      </c>
-      <c r="E5" t="n">
-        <v>104.331</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>A05,A06</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>#13 1NM</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2</v>
-      </c>
-      <c r="C6" t="n">
-        <v>2</v>
-      </c>
-      <c r="D6" t="n">
-        <v>1829.2</v>
-      </c>
-      <c r="E6" t="n">
-        <v>62.859</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>A07,A08</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>#13 0,5NM</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>1</v>
-      </c>
-      <c r="C7" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" t="n">
-        <v>1366.621</v>
-      </c>
-      <c r="E7" t="n">
-        <v>76.241</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>A09,A10</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>#13 0,5NM</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2</v>
-      </c>
-      <c r="C8" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" t="n">
-        <v>1737.055</v>
-      </c>
-      <c r="E8" t="n">
-        <v>194.166</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>A11,A12</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Sin corregir · por condición (media ± SD de las 2 biológicas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Condicion</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>sd</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>minimo</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>maximo</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>c-</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2</v>
-      </c>
-      <c r="C12" t="n">
-        <v>2214.085</v>
-      </c>
-      <c r="D12" t="n">
-        <v>417.056</v>
-      </c>
-      <c r="E12" t="n">
-        <v>1919.182</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2508.988</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>#13 0,5NM</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>2</v>
-      </c>
-      <c r="C13" t="n">
-        <v>1551.838</v>
-      </c>
-      <c r="D13" t="n">
-        <v>261.936</v>
-      </c>
-      <c r="E13" t="n">
-        <v>1366.621</v>
-      </c>
-      <c r="F13" t="n">
-        <v>1737.055</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>#13 1NM</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C14" t="n">
-        <v>1268.225</v>
-      </c>
-      <c r="D14" t="n">
-        <v>793.338</v>
-      </c>
-      <c r="E14" t="n">
-        <v>707.25</v>
-      </c>
-      <c r="F14" t="n">
-        <v>1829.2</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Corregido por RNA · por réplica biológica (media de las técnicas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Condicion</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Rep_bio</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>n_tecnicas</t>
-        </is>
-      </c>
-      <c r="D17" s="4" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>sd_tecnica</t>
-        </is>
-      </c>
-      <c r="F17" s="4" t="inlineStr">
-        <is>
-          <t>pocillos</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>c-</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>1</v>
-      </c>
-      <c r="C18" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" t="n">
-        <v>3584.269</v>
-      </c>
-      <c r="E18" t="n">
-        <v>118.67</v>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>A01,A02</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>c-</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>2</v>
-      </c>
-      <c r="C19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" t="n">
-        <v>3095.455</v>
-      </c>
-      <c r="E19" t="n">
-        <v>180.327</v>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>A03,A04</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>#13 1NM</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
-      </c>
-      <c r="C20" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" t="n">
-        <v>1360.097</v>
-      </c>
-      <c r="E20" t="n">
-        <v>200.637</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>A05,A06</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>#13 1NM</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>2</v>
-      </c>
-      <c r="C21" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" t="n">
-        <v>2286.5</v>
-      </c>
-      <c r="E21" t="n">
-        <v>78.574</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>A07,A08</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>#13 0,5NM</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>1</v>
-      </c>
-      <c r="C22" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" t="n">
-        <v>2628.117</v>
-      </c>
-      <c r="E22" t="n">
-        <v>146.617</v>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>A09,A10</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>#13 0,5NM</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>2</v>
-      </c>
-      <c r="C23" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" t="n">
-        <v>2198.804</v>
-      </c>
-      <c r="E23" t="n">
-        <v>245.78</v>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>A11,A12</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Corregido por RNA · por condición (media ± SD de las 2 biológicas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Condicion</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
-        <is>
-          <t>media</t>
-        </is>
-      </c>
-      <c r="D26" s="4" t="inlineStr">
-        <is>
-          <t>sd</t>
-        </is>
-      </c>
-      <c r="E26" s="4" t="inlineStr">
-        <is>
-          <t>minimo</t>
-        </is>
-      </c>
-      <c r="F26" s="4" t="inlineStr">
-        <is>
-          <t>maximo</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>c-</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>2</v>
-      </c>
-      <c r="C27" t="n">
-        <v>3339.862</v>
-      </c>
-      <c r="D27" t="n">
-        <v>345.644</v>
-      </c>
-      <c r="E27" t="n">
-        <v>3095.455</v>
-      </c>
-      <c r="F27" t="n">
-        <v>3584.269</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>#13 0,5NM</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>2</v>
-      </c>
-      <c r="C28" t="n">
-        <v>2413.46</v>
-      </c>
-      <c r="D28" t="n">
-        <v>303.57</v>
-      </c>
-      <c r="E28" t="n">
-        <v>2198.804</v>
-      </c>
-      <c r="F28" t="n">
-        <v>2628.117</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>#13 1NM</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>2</v>
-      </c>
-      <c r="C29" t="n">
-        <v>1823.299</v>
-      </c>
-      <c r="D29" t="n">
-        <v>655.066</v>
-      </c>
-      <c r="E29" t="n">
-        <v>1360.097</v>
-      </c>
-      <c r="F29" t="n">
-        <v>2286.5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>